<commit_message>
Corrige comparativo: NF 3561 na lista do usuário é 13%, não 47%
Erro no registro da lista; 3561 confere com o dashboard (~13,1%).

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Lista_vs_Dashboard_Jul.xlsx
+++ b/Comparacao_Lista_vs_Dashboard_Jul.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,7 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Δ pp (lista−dash)</t>
+          <t>Δ pp</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -449,20 +449,25 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Venda dash</t>
+          <t>Obs</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Custo dash</t>
+          <t>Venda</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Frete dash</t>
+          <t>Custo</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
+        <is>
+          <t>Frete</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Itens</t>
         </is>
@@ -475,7 +480,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="C2" t="n">
         <v>13.12</v>
@@ -484,23 +489,28 @@
         <v>13.12</v>
       </c>
       <c r="E2" t="n">
-        <v>33.88</v>
+        <v>0.12</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+          <t>CONFERE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Lista corrigida para 13% (antes constava 47% por erro)</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
         <v>525.6</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>360</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>70</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -527,16 +537,17 @@
           <t>CONFERE</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
         <v>1348.56</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>806.4</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>57.74</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -560,9 +571,8 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -587,16 +597,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
         <v>645.36</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>343.2</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -620,9 +631,8 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="n">
-        <v>1</v>
-      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -645,6 +655,7 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -669,16 +680,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
         <v>1007.76</v>
       </c>
-      <c r="H8" t="n">
+      <c r="I8" t="n">
         <v>603.5999999999999</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>101.61</v>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>2</v>
       </c>
     </row>
@@ -705,16 +717,17 @@
           <t>CONFERE</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
         <v>560.8</v>
       </c>
-      <c r="H9" t="n">
+      <c r="I9" t="n">
         <v>332</v>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>25</v>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -741,16 +754,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
         <v>1188</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>547.6799999999999</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>153.14</v>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -777,16 +791,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
         <v>74.59999999999999</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>18.58</v>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>25</v>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>1</v>
       </c>
     </row>
@@ -811,6 +826,7 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -833,16 +849,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G13" t="n">
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
         <v>3486.7</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>2795.77</v>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>0</v>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -867,16 +884,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G14" t="n">
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
         <v>718.5599999999999</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>475.2</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="J14" t="n">
+      <c r="K14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -903,16 +921,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G15" t="n">
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
         <v>2102.4</v>
       </c>
-      <c r="H15" t="n">
+      <c r="I15" t="n">
         <v>1440</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>120</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -939,16 +958,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G16" t="n">
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
         <v>718.5599999999999</v>
       </c>
-      <c r="H16" t="n">
+      <c r="I16" t="n">
         <v>475.2</v>
       </c>
-      <c r="I16" t="n">
+      <c r="J16" t="n">
         <v>60</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -973,6 +993,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -997,16 +1018,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G18" t="n">
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
         <v>19820</v>
       </c>
-      <c r="H18" t="n">
+      <c r="I18" t="n">
         <v>12595</v>
       </c>
-      <c r="I18" t="n">
+      <c r="J18" t="n">
         <v>190</v>
       </c>
-      <c r="J18" t="n">
+      <c r="K18" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1033,16 +1055,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
         <v>2874.24</v>
       </c>
-      <c r="H19" t="n">
+      <c r="I19" t="n">
         <v>1900.8</v>
       </c>
-      <c r="I19" t="n">
+      <c r="J19" t="n">
         <v>60</v>
       </c>
-      <c r="J19" t="n">
+      <c r="K19" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1069,16 +1092,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G20" t="n">
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
         <v>3374.5</v>
       </c>
-      <c r="H20" t="n">
+      <c r="I20" t="n">
         <v>1869.94</v>
       </c>
-      <c r="I20" t="n">
+      <c r="J20" t="n">
         <v>40</v>
       </c>
-      <c r="J20" t="n">
+      <c r="K20" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1105,16 +1129,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G21" t="n">
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
         <v>292.8</v>
       </c>
-      <c r="H21" t="n">
+      <c r="I21" t="n">
         <v>127.68</v>
       </c>
-      <c r="I21" t="n">
+      <c r="J21" t="n">
         <v>0</v>
       </c>
-      <c r="J21" t="n">
+      <c r="K21" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1141,16 +1166,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
         <v>376</v>
       </c>
-      <c r="H22" t="n">
+      <c r="I22" t="n">
         <v>133</v>
       </c>
-      <c r="I22" t="n">
+      <c r="J22" t="n">
         <v>59</v>
       </c>
-      <c r="J22" t="n">
+      <c r="K22" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1177,16 +1203,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G23" t="n">
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
         <v>460</v>
       </c>
-      <c r="H23" t="n">
+      <c r="I23" t="n">
         <v>266</v>
       </c>
-      <c r="I23" t="n">
+      <c r="J23" t="n">
         <v>47.81</v>
       </c>
-      <c r="J23" t="n">
+      <c r="K23" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1213,16 +1240,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G24" t="n">
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
         <v>3316</v>
       </c>
-      <c r="H24" t="n">
+      <c r="I24" t="n">
         <v>2253.38</v>
       </c>
-      <c r="I24" t="n">
+      <c r="J24" t="n">
         <v>0</v>
       </c>
-      <c r="J24" t="n">
+      <c r="K24" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1249,16 +1277,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G25" t="n">
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
         <v>556</v>
       </c>
-      <c r="H25" t="n">
+      <c r="I25" t="n">
         <v>228.2</v>
       </c>
-      <c r="I25" t="n">
+      <c r="J25" t="n">
         <v>40</v>
       </c>
-      <c r="J25" t="n">
+      <c r="K25" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1285,16 +1314,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
         <v>1820</v>
       </c>
-      <c r="H26" t="n">
+      <c r="I26" t="n">
         <v>1162</v>
       </c>
-      <c r="I26" t="n">
+      <c r="J26" t="n">
         <v>30</v>
       </c>
-      <c r="J26" t="n">
+      <c r="K26" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1321,16 +1351,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G27" t="n">
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
         <v>704.7</v>
       </c>
-      <c r="H27" t="n">
+      <c r="I27" t="n">
         <v>288.3</v>
       </c>
-      <c r="I27" t="n">
+      <c r="J27" t="n">
         <v>50</v>
       </c>
-      <c r="J27" t="n">
+      <c r="K27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1355,16 +1386,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G28" t="n">
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
         <v>1277</v>
       </c>
-      <c r="H28" t="n">
+      <c r="I28" t="n">
         <v>998.3200000000001</v>
       </c>
-      <c r="I28" t="n">
+      <c r="J28" t="n">
         <v>0</v>
       </c>
-      <c r="J28" t="n">
+      <c r="K28" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1391,16 +1423,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G29" t="n">
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
         <v>10590</v>
       </c>
-      <c r="H29" t="n">
+      <c r="I29" t="n">
         <v>7834.799999999999</v>
       </c>
-      <c r="I29" t="n">
+      <c r="J29" t="n">
         <v>0</v>
       </c>
-      <c r="J29" t="n">
+      <c r="K29" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1427,16 +1460,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G30" t="n">
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
         <v>928.36</v>
       </c>
-      <c r="H30" t="n">
+      <c r="I30" t="n">
         <v>534</v>
       </c>
-      <c r="I30" t="n">
+      <c r="J30" t="n">
         <v>60</v>
       </c>
-      <c r="J30" t="n">
+      <c r="K30" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1463,16 +1497,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G31" t="n">
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
         <v>1485</v>
       </c>
-      <c r="H31" t="n">
+      <c r="I31" t="n">
         <v>684.6</v>
       </c>
-      <c r="I31" t="n">
+      <c r="J31" t="n">
         <v>137.74</v>
       </c>
-      <c r="J31" t="n">
+      <c r="K31" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1499,16 +1534,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G32" t="n">
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="n">
         <v>1137.12</v>
       </c>
-      <c r="H32" t="n">
+      <c r="I32" t="n">
         <v>686.4</v>
       </c>
-      <c r="I32" t="n">
+      <c r="J32" t="n">
         <v>60</v>
       </c>
-      <c r="J32" t="n">
+      <c r="K32" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1533,16 +1569,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G33" t="n">
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="n">
         <v>1017.2</v>
       </c>
-      <c r="H33" t="n">
+      <c r="I33" t="n">
         <v>578.59</v>
       </c>
-      <c r="I33" t="n">
+      <c r="J33" t="n">
         <v>59.34</v>
       </c>
-      <c r="J33" t="n">
+      <c r="K33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1569,16 +1606,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G34" t="n">
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="n">
         <v>1673.28</v>
       </c>
-      <c r="H34" t="n">
+      <c r="I34" t="n">
         <v>760.3200000000001</v>
       </c>
-      <c r="I34" t="n">
+      <c r="J34" t="n">
         <v>300</v>
       </c>
-      <c r="J34" t="n">
+      <c r="K34" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1605,16 +1643,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G35" t="n">
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="n">
         <v>1673.28</v>
       </c>
-      <c r="H35" t="n">
+      <c r="I35" t="n">
         <v>760.3200000000001</v>
       </c>
-      <c r="I35" t="n">
+      <c r="J35" t="n">
         <v>199.5</v>
       </c>
-      <c r="J35" t="n">
+      <c r="K35" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1639,16 +1678,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G36" t="n">
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="n">
         <v>1044.2</v>
       </c>
-      <c r="H36" t="n">
+      <c r="I36" t="n">
         <v>679.3399999999999</v>
       </c>
-      <c r="I36" t="n">
+      <c r="J36" t="n">
         <v>45</v>
       </c>
-      <c r="J36" t="n">
+      <c r="K36" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1675,16 +1715,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G37" t="n">
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="n">
         <v>645.36</v>
       </c>
-      <c r="H37" t="n">
+      <c r="I37" t="n">
         <v>343.2</v>
       </c>
-      <c r="I37" t="n">
+      <c r="J37" t="n">
         <v>0</v>
       </c>
-      <c r="J37" t="n">
+      <c r="K37" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1711,16 +1752,17 @@
           <t>DIVERGE</t>
         </is>
       </c>
-      <c r="G38" t="n">
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="n">
         <v>1372.5</v>
       </c>
-      <c r="H38" t="n">
+      <c r="I38" t="n">
         <v>674.13</v>
       </c>
-      <c r="I38" t="n">
+      <c r="J38" t="n">
         <v>219.41</v>
       </c>
-      <c r="J38" t="n">
+      <c r="K38" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1747,16 +1789,17 @@
           <t>CONFERE</t>
         </is>
       </c>
-      <c r="G39" t="n">
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="n">
         <v>2352</v>
       </c>
-      <c r="H39" t="n">
+      <c r="I39" t="n">
         <v>1372.8</v>
       </c>
-      <c r="I39" t="n">
+      <c r="J39" t="n">
         <v>120</v>
       </c>
-      <c r="J39" t="n">
+      <c r="K39" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Exclui NF 3563 do relatório e do dashboard
Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Lista_vs_Dashboard_Jul.xlsx
+++ b/Comparacao_Lista_vs_Dashboard_Jul.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,10 +474,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>3561</t>
-        </is>
+      <c r="A2" t="n">
+        <v>3561</v>
       </c>
       <c r="B2" t="n">
         <v>13</v>
@@ -515,10 +513,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>3562</t>
-        </is>
+      <c r="A3" t="n">
+        <v>3562</v>
       </c>
       <c r="B3" t="n">
         <v>45</v>
@@ -552,80 +548,74 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3563</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3564</v>
       </c>
       <c r="B4" t="n">
-        <v>42</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+        <v>39</v>
+      </c>
+      <c r="C4" t="n">
+        <v>70.73999999999999</v>
+      </c>
+      <c r="D4" t="n">
+        <v>70.73999999999999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>31.74</v>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>DIVERGE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>645.36</v>
+      </c>
+      <c r="I4" t="n">
+        <v>343.2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3565</v>
+      </c>
+      <c r="B5" t="n">
+        <v>55</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>SEM_CUSTO</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>3564</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>39</v>
-      </c>
-      <c r="C5" t="n">
-        <v>70.73999999999999</v>
-      </c>
-      <c r="D5" t="n">
-        <v>70.73999999999999</v>
-      </c>
-      <c r="E5" t="n">
-        <v>31.74</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>DIVERGE</t>
-        </is>
-      </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>645.36</v>
-      </c>
-      <c r="I5" t="n">
-        <v>343.2</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>3565</t>
-        </is>
+      <c r="A6" t="n">
+        <v>3566</v>
       </c>
       <c r="B6" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SEM_CUSTO</t>
+          <t>CANCELADA</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -635,119 +625,125 @@
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3566</t>
-        </is>
+      <c r="A7" t="n">
+        <v>3567</v>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="C7" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="D7" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="E7" t="n">
+        <v>25.24</v>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CANCELADA</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>1007.76</v>
+      </c>
+      <c r="I7" t="n">
+        <v>603.5999999999999</v>
+      </c>
+      <c r="J7" t="n">
+        <v>101.61</v>
+      </c>
+      <c r="K7" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>3567</t>
-        </is>
+      <c r="A8" t="n">
+        <v>3568</v>
       </c>
       <c r="B8" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="C8" t="n">
-        <v>34.76</v>
+        <v>45.85</v>
       </c>
       <c r="D8" t="n">
-        <v>34.76</v>
+        <v>45.85</v>
       </c>
       <c r="E8" t="n">
-        <v>25.24</v>
+        <v>0.15</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>CONFERE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>1007.76</v>
+        <v>560.8</v>
       </c>
       <c r="I8" t="n">
-        <v>603.5999999999999</v>
+        <v>332</v>
       </c>
       <c r="J8" t="n">
-        <v>101.61</v>
+        <v>25</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>3568</t>
-        </is>
+      <c r="A9" t="n">
+        <v>3569</v>
       </c>
       <c r="B9" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="C9" t="n">
-        <v>45.85</v>
+        <v>69</v>
       </c>
       <c r="D9" t="n">
-        <v>45.85</v>
+        <v>69</v>
       </c>
       <c r="E9" t="n">
-        <v>0.15</v>
+        <v>7</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CONFERE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>560.8</v>
+        <v>1188</v>
       </c>
       <c r="I9" t="n">
-        <v>332</v>
+        <v>547.6799999999999</v>
       </c>
       <c r="J9" t="n">
-        <v>25</v>
+        <v>153.14</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>3569</t>
-        </is>
+      <c r="A10" t="n">
+        <v>3570</v>
       </c>
       <c r="B10" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>69</v>
+        <v>130.02</v>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>130.02</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>100.02</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -756,93 +752,85 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>1188</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>547.6799999999999</v>
+        <v>18.58</v>
       </c>
       <c r="J10" t="n">
-        <v>153.14</v>
+        <v>25</v>
       </c>
       <c r="K10" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>3570</t>
-        </is>
+      <c r="A11" t="n">
+        <v>3571</v>
       </c>
       <c r="B11" t="n">
-        <v>30</v>
-      </c>
-      <c r="C11" t="n">
-        <v>130.02</v>
-      </c>
-      <c r="D11" t="n">
-        <v>130.02</v>
-      </c>
-      <c r="E11" t="n">
-        <v>100.02</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>AUSENTE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="I11" t="n">
-        <v>18.58</v>
-      </c>
-      <c r="J11" t="n">
-        <v>25</v>
-      </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>3571</t>
-        </is>
+      <c r="A12" t="n">
+        <v>3572</v>
       </c>
       <c r="B12" t="n">
-        <v>31</v>
-      </c>
-      <c r="C12" t="inlineStr"/>
+        <v>41</v>
+      </c>
+      <c r="C12" t="n">
+        <v>13.24</v>
+      </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>27.76</v>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AUSENTE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>3486.7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2795.77</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>3572</t>
-        </is>
+      <c r="A13" t="n">
+        <v>3573</v>
       </c>
       <c r="B13" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C13" t="n">
-        <v>13.24</v>
+        <v>37.3</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>27.76</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -851,10 +839,10 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>3486.7</v>
+        <v>718.5599999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>2795.77</v>
+        <v>475.2</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -864,20 +852,20 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>3573</t>
-        </is>
+      <c r="A14" t="n">
+        <v>3574</v>
       </c>
       <c r="B14" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C14" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="D14" t="inlineStr"/>
+        <v>24.23</v>
+      </c>
+      <c r="D14" t="n">
+        <v>24.23</v>
+      </c>
       <c r="E14" t="n">
-        <v>9.699999999999999</v>
+        <v>19.77</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -886,35 +874,33 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>718.5599999999999</v>
+        <v>2102.4</v>
       </c>
       <c r="I14" t="n">
-        <v>475.2</v>
+        <v>1440</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="K14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>3574</t>
-        </is>
+      <c r="A15" t="n">
+        <v>3575</v>
       </c>
       <c r="B15" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C15" t="n">
-        <v>24.23</v>
+        <v>24.67</v>
       </c>
       <c r="D15" t="n">
-        <v>24.23</v>
+        <v>24.67</v>
       </c>
       <c r="E15" t="n">
-        <v>19.77</v>
+        <v>33.33</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -923,95 +909,89 @@
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>2102.4</v>
+        <v>718.5599999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>1440</v>
+        <v>475.2</v>
       </c>
       <c r="J15" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="K15" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>3575</t>
-        </is>
+      <c r="A16" t="n">
+        <v>3576</v>
       </c>
       <c r="B16" t="n">
-        <v>58</v>
-      </c>
-      <c r="C16" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="D16" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="E16" t="n">
-        <v>33.33</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>AUSENTE</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="n">
-        <v>718.5599999999999</v>
-      </c>
-      <c r="I16" t="n">
-        <v>475.2</v>
-      </c>
-      <c r="J16" t="n">
-        <v>60</v>
-      </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>3576</t>
-        </is>
+      <c r="A17" t="n">
+        <v>3577</v>
       </c>
       <c r="B17" t="n">
-        <v>48</v>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+        <v>46</v>
+      </c>
+      <c r="C17" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="D17" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4.62</v>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AUSENTE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>19820</v>
+      </c>
+      <c r="I17" t="n">
+        <v>12595</v>
+      </c>
+      <c r="J17" t="n">
+        <v>190</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>3577</t>
-        </is>
+      <c r="A18" t="n">
+        <v>3578</v>
       </c>
       <c r="B18" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C18" t="n">
-        <v>41.38</v>
+        <v>34.14</v>
       </c>
       <c r="D18" t="n">
-        <v>41.38</v>
+        <v>34.14</v>
       </c>
       <c r="E18" t="n">
-        <v>4.62</v>
+        <v>18.86</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1020,35 +1000,33 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>19820</v>
+        <v>2874.24</v>
       </c>
       <c r="I18" t="n">
-        <v>12595</v>
+        <v>1900.8</v>
       </c>
       <c r="J18" t="n">
-        <v>190</v>
+        <v>60</v>
       </c>
       <c r="K18" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>3578</t>
-        </is>
+      <c r="A19" t="n">
+        <v>3579</v>
       </c>
       <c r="B19" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C19" t="n">
-        <v>34.14</v>
+        <v>61.72</v>
       </c>
       <c r="D19" t="n">
-        <v>34.14</v>
+        <v>51.75</v>
       </c>
       <c r="E19" t="n">
-        <v>18.86</v>
+        <v>11.72</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1057,35 +1035,33 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>2874.24</v>
+        <v>3374.5</v>
       </c>
       <c r="I19" t="n">
-        <v>1900.8</v>
+        <v>1869.94</v>
       </c>
       <c r="J19" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>3579</t>
-        </is>
+      <c r="A20" t="n">
+        <v>3580</v>
       </c>
       <c r="B20" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C20" t="n">
-        <v>61.72</v>
+        <v>108.23</v>
       </c>
       <c r="D20" t="n">
-        <v>51.75</v>
+        <v>108.23</v>
       </c>
       <c r="E20" t="n">
-        <v>11.72</v>
+        <v>62.23</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1094,35 +1070,33 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>3374.5</v>
+        <v>292.8</v>
       </c>
       <c r="I20" t="n">
-        <v>1869.94</v>
+        <v>127.68</v>
       </c>
       <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3581</v>
+      </c>
+      <c r="B21" t="n">
         <v>40</v>
       </c>
-      <c r="K20" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>3580</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>46</v>
-      </c>
       <c r="C21" t="n">
-        <v>108.23</v>
+        <v>112.34</v>
       </c>
       <c r="D21" t="n">
-        <v>108.23</v>
+        <v>112.34</v>
       </c>
       <c r="E21" t="n">
-        <v>62.23</v>
+        <v>72.34</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1131,35 +1105,33 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>292.8</v>
+        <v>376</v>
       </c>
       <c r="I21" t="n">
-        <v>127.68</v>
+        <v>133</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="K21" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>3581</t>
-        </is>
+      <c r="A22" t="n">
+        <v>3582</v>
       </c>
       <c r="B22" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C22" t="n">
-        <v>112.34</v>
+        <v>39.05</v>
       </c>
       <c r="D22" t="n">
-        <v>112.34</v>
+        <v>39.05</v>
       </c>
       <c r="E22" t="n">
-        <v>72.34</v>
+        <v>12.95</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1168,35 +1140,33 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>376</v>
+        <v>460</v>
       </c>
       <c r="I22" t="n">
-        <v>133</v>
+        <v>266</v>
       </c>
       <c r="J22" t="n">
-        <v>59</v>
+        <v>47.81</v>
       </c>
       <c r="K22" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>3582</t>
-        </is>
+      <c r="A23" t="n">
+        <v>3583</v>
       </c>
       <c r="B23" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C23" t="n">
-        <v>39.05</v>
+        <v>33.62</v>
       </c>
       <c r="D23" t="n">
-        <v>39.05</v>
+        <v>18.71</v>
       </c>
       <c r="E23" t="n">
-        <v>12.95</v>
+        <v>13.38</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1205,35 +1175,33 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>460</v>
+        <v>3316</v>
       </c>
       <c r="I23" t="n">
-        <v>266</v>
+        <v>2253.38</v>
       </c>
       <c r="J23" t="n">
-        <v>47.81</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>3583</t>
-        </is>
+      <c r="A24" t="n">
+        <v>3584</v>
       </c>
       <c r="B24" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C24" t="n">
-        <v>33.62</v>
+        <v>103.7</v>
       </c>
       <c r="D24" t="n">
-        <v>18.71</v>
+        <v>103.7</v>
       </c>
       <c r="E24" t="n">
-        <v>13.38</v>
+        <v>49.7</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1242,35 +1210,33 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>3316</v>
+        <v>556</v>
       </c>
       <c r="I24" t="n">
-        <v>2253.38</v>
+        <v>228.2</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="K24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>3584</t>
-        </is>
+      <c r="A25" t="n">
+        <v>3585</v>
       </c>
       <c r="B25" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C25" t="n">
-        <v>103.7</v>
+        <v>39.64</v>
       </c>
       <c r="D25" t="n">
-        <v>103.7</v>
+        <v>39.64</v>
       </c>
       <c r="E25" t="n">
-        <v>49.7</v>
+        <v>16.36</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1279,35 +1245,33 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>556</v>
+        <v>1820</v>
       </c>
       <c r="I25" t="n">
-        <v>228.2</v>
+        <v>1162</v>
       </c>
       <c r="J25" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>3585</t>
-        </is>
+      <c r="A26" t="n">
+        <v>3586</v>
       </c>
       <c r="B26" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C26" t="n">
-        <v>39.64</v>
+        <v>104.6</v>
       </c>
       <c r="D26" t="n">
-        <v>39.64</v>
+        <v>104.6</v>
       </c>
       <c r="E26" t="n">
-        <v>16.36</v>
+        <v>57.6</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1316,35 +1280,31 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>1820</v>
+        <v>704.7</v>
       </c>
       <c r="I26" t="n">
-        <v>1162</v>
+        <v>288.3</v>
       </c>
       <c r="J26" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>3586</t>
-        </is>
+      <c r="A27" t="n">
+        <v>3587</v>
       </c>
       <c r="B27" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C27" t="n">
-        <v>104.6</v>
-      </c>
-      <c r="D27" t="n">
-        <v>104.6</v>
-      </c>
+        <v>16.15</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>57.6</v>
+        <v>28.85</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1353,33 +1313,33 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>704.7</v>
+        <v>1277</v>
       </c>
       <c r="I27" t="n">
-        <v>288.3</v>
+        <v>998.3200000000001</v>
       </c>
       <c r="J27" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>3587</t>
-        </is>
+      <c r="A28" t="n">
+        <v>3588</v>
       </c>
       <c r="B28" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C28" t="n">
-        <v>16.15</v>
-      </c>
-      <c r="D28" t="inlineStr"/>
+        <v>22.73</v>
+      </c>
+      <c r="D28" t="n">
+        <v>40.38</v>
+      </c>
       <c r="E28" t="n">
-        <v>28.85</v>
+        <v>38.27</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1388,35 +1348,33 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>1277</v>
+        <v>10590</v>
       </c>
       <c r="I28" t="n">
-        <v>998.3200000000001</v>
+        <v>7834.799999999999</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>3588</t>
-        </is>
+      <c r="A29" t="n">
+        <v>3589</v>
       </c>
       <c r="B29" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C29" t="n">
-        <v>22.73</v>
+        <v>46.62</v>
       </c>
       <c r="D29" t="n">
-        <v>40.38</v>
+        <v>46.62</v>
       </c>
       <c r="E29" t="n">
-        <v>38.27</v>
+        <v>11.62</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1425,35 +1383,33 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>10590</v>
+        <v>928.36</v>
       </c>
       <c r="I29" t="n">
-        <v>7834.799999999999</v>
+        <v>534</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>3589</t>
-        </is>
+      <c r="A30" t="n">
+        <v>3590</v>
       </c>
       <c r="B30" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C30" t="n">
-        <v>46.62</v>
+        <v>76.84</v>
       </c>
       <c r="D30" t="n">
-        <v>46.62</v>
+        <v>76.84</v>
       </c>
       <c r="E30" t="n">
-        <v>11.62</v>
+        <v>32.84</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1462,35 +1418,33 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>928.36</v>
+        <v>1485</v>
       </c>
       <c r="I30" t="n">
-        <v>534</v>
+        <v>684.6</v>
       </c>
       <c r="J30" t="n">
-        <v>60</v>
+        <v>137.74</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>3590</t>
-        </is>
+      <c r="A31" t="n">
+        <v>3591</v>
       </c>
       <c r="B31" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C31" t="n">
-        <v>76.84</v>
+        <v>41.68</v>
       </c>
       <c r="D31" t="n">
-        <v>76.84</v>
+        <v>41.68</v>
       </c>
       <c r="E31" t="n">
-        <v>32.84</v>
+        <v>3.32</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1499,35 +1453,31 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>1485</v>
+        <v>1137.12</v>
       </c>
       <c r="I31" t="n">
-        <v>684.6</v>
+        <v>686.4</v>
       </c>
       <c r="J31" t="n">
-        <v>137.74</v>
+        <v>60</v>
       </c>
       <c r="K31" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>3591</t>
-        </is>
+      <c r="A32" t="n">
+        <v>3592</v>
       </c>
       <c r="B32" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C32" t="n">
-        <v>41.68</v>
-      </c>
-      <c r="D32" t="n">
-        <v>41.68</v>
-      </c>
+        <v>49.38</v>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>3.32</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1536,33 +1486,33 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>1137.12</v>
+        <v>1017.2</v>
       </c>
       <c r="I32" t="n">
-        <v>686.4</v>
+        <v>578.59</v>
       </c>
       <c r="J32" t="n">
-        <v>60</v>
+        <v>59.34</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>3592</t>
-        </is>
+      <c r="A33" t="n">
+        <v>3593</v>
       </c>
       <c r="B33" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C33" t="n">
-        <v>49.38</v>
-      </c>
-      <c r="D33" t="inlineStr"/>
+        <v>60.37</v>
+      </c>
+      <c r="D33" t="n">
+        <v>60.37</v>
+      </c>
       <c r="E33" t="n">
-        <v>9.380000000000001</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1571,35 +1521,33 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>1017.2</v>
+        <v>1673.28</v>
       </c>
       <c r="I33" t="n">
-        <v>578.59</v>
+        <v>760.3200000000001</v>
       </c>
       <c r="J33" t="n">
-        <v>59.34</v>
+        <v>300</v>
       </c>
       <c r="K33" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>3593</t>
-        </is>
+      <c r="A34" t="n">
+        <v>3594</v>
       </c>
       <c r="B34" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C34" t="n">
-        <v>60.37</v>
+        <v>73.59</v>
       </c>
       <c r="D34" t="n">
-        <v>60.37</v>
+        <v>73.59</v>
       </c>
       <c r="E34" t="n">
-        <v>8.369999999999999</v>
+        <v>26.59</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1614,29 +1562,25 @@
         <v>760.3200000000001</v>
       </c>
       <c r="J34" t="n">
-        <v>300</v>
+        <v>199.5</v>
       </c>
       <c r="K34" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>3594</t>
-        </is>
+      <c r="A35" t="n">
+        <v>3595</v>
       </c>
       <c r="B35" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C35" t="n">
-        <v>73.59</v>
-      </c>
-      <c r="D35" t="n">
-        <v>73.59</v>
-      </c>
+        <v>32.94</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="n">
-        <v>26.59</v>
+        <v>6.06</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1645,33 +1589,33 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>1673.28</v>
+        <v>1044.2</v>
       </c>
       <c r="I35" t="n">
-        <v>760.3200000000001</v>
+        <v>679.3399999999999</v>
       </c>
       <c r="J35" t="n">
-        <v>199.5</v>
+        <v>45</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>3595</t>
-        </is>
+      <c r="A36" t="n">
+        <v>3596</v>
       </c>
       <c r="B36" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C36" t="n">
-        <v>32.94</v>
-      </c>
-      <c r="D36" t="inlineStr"/>
+        <v>70.73999999999999</v>
+      </c>
+      <c r="D36" t="n">
+        <v>70.73999999999999</v>
+      </c>
       <c r="E36" t="n">
-        <v>6.06</v>
+        <v>26.74</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1680,35 +1624,33 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>1044.2</v>
+        <v>645.36</v>
       </c>
       <c r="I36" t="n">
-        <v>679.3399999999999</v>
+        <v>343.2</v>
       </c>
       <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>3597</v>
+      </c>
+      <c r="B37" t="n">
         <v>45</v>
       </c>
-      <c r="K36" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>3596</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>44</v>
-      </c>
       <c r="C37" t="n">
-        <v>70.73999999999999</v>
+        <v>52.32</v>
       </c>
       <c r="D37" t="n">
-        <v>70.73999999999999</v>
+        <v>52.32</v>
       </c>
       <c r="E37" t="n">
-        <v>26.74</v>
+        <v>7.32</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1717,89 +1659,50 @@
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>645.36</v>
+        <v>1372.5</v>
       </c>
       <c r="I37" t="n">
-        <v>343.2</v>
+        <v>674.13</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>219.41</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>3597</t>
-        </is>
+      <c r="A38" t="n">
+        <v>3598</v>
       </c>
       <c r="B38" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C38" t="n">
-        <v>52.32</v>
+        <v>46.83</v>
       </c>
       <c r="D38" t="n">
-        <v>52.32</v>
+        <v>46.83</v>
       </c>
       <c r="E38" t="n">
-        <v>7.32</v>
+        <v>0.17</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>CONFERE</t>
         </is>
       </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
-        <v>1372.5</v>
+        <v>2352</v>
       </c>
       <c r="I38" t="n">
-        <v>674.13</v>
+        <v>1372.8</v>
       </c>
       <c r="J38" t="n">
-        <v>219.41</v>
+        <v>120</v>
       </c>
       <c r="K38" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>3598</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>47</v>
-      </c>
-      <c r="C39" t="n">
-        <v>46.83</v>
-      </c>
-      <c r="D39" t="n">
-        <v>46.83</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>CONFERE</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="n">
-        <v>2352</v>
-      </c>
-      <c r="I39" t="n">
-        <v>1372.8</v>
-      </c>
-      <c r="J39" t="n">
-        <v>120</v>
-      </c>
-      <c r="K39" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige comparativo: NF 3564 na lista do usuário é 70,74%, não 39%
Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Lista_vs_Dashboard_Jul.xlsx
+++ b/Comparacao_Lista_vs_Dashboard_Jul.xlsx
@@ -474,8 +474,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>3561</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>3561</t>
+        </is>
       </c>
       <c r="B2" t="n">
         <v>13</v>
@@ -496,7 +498,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Lista corrigida para 13% (antes constava 47% por erro)</t>
+          <t>Lista 13% (corrigido)</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -513,8 +515,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>3562</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3562</t>
+        </is>
       </c>
       <c r="B3" t="n">
         <v>45</v>
@@ -548,11 +552,13 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3564</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3564</t>
+        </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>70.73999999999999</v>
       </c>
       <c r="C4" t="n">
         <v>70.73999999999999</v>
@@ -561,14 +567,18 @@
         <v>70.73999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>31.74</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>CONFERE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Lista 70,74% (corrigido; antes constava 39% por erro)</t>
+        </is>
+      </c>
       <c r="H4" t="n">
         <v>645.36</v>
       </c>
@@ -583,8 +593,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>3565</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3565</t>
+        </is>
       </c>
       <c r="B5" t="n">
         <v>55</v>
@@ -604,8 +616,10 @@
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>3566</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3566</t>
+        </is>
       </c>
       <c r="B6" t="n">
         <v>48</v>
@@ -625,8 +639,10 @@
       <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>3567</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3567</t>
+        </is>
       </c>
       <c r="B7" t="n">
         <v>60</v>
@@ -660,8 +676,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>3568</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3568</t>
+        </is>
       </c>
       <c r="B8" t="n">
         <v>46</v>
@@ -695,8 +713,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>3569</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>3569</t>
+        </is>
       </c>
       <c r="B9" t="n">
         <v>62</v>
@@ -730,8 +750,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>3570</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>3570</t>
+        </is>
       </c>
       <c r="B10" t="n">
         <v>30</v>
@@ -765,8 +787,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>3571</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3571</t>
+        </is>
       </c>
       <c r="B11" t="n">
         <v>31</v>
@@ -786,8 +810,10 @@
       <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>3572</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3572</t>
+        </is>
       </c>
       <c r="B12" t="n">
         <v>41</v>
@@ -819,8 +845,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>3573</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3573</t>
+        </is>
       </c>
       <c r="B13" t="n">
         <v>47</v>
@@ -852,8 +880,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>3574</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>3574</t>
+        </is>
       </c>
       <c r="B14" t="n">
         <v>44</v>
@@ -887,8 +917,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>3575</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3575</t>
+        </is>
       </c>
       <c r="B15" t="n">
         <v>58</v>
@@ -922,8 +954,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>3576</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>3576</t>
+        </is>
       </c>
       <c r="B16" t="n">
         <v>48</v>
@@ -943,8 +977,10 @@
       <c r="K16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>3577</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>3577</t>
+        </is>
       </c>
       <c r="B17" t="n">
         <v>46</v>
@@ -978,8 +1014,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>3578</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3578</t>
+        </is>
       </c>
       <c r="B18" t="n">
         <v>53</v>
@@ -1013,8 +1051,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>3579</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3579</t>
+        </is>
       </c>
       <c r="B19" t="n">
         <v>50</v>
@@ -1048,8 +1088,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>3580</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>3580</t>
+        </is>
       </c>
       <c r="B20" t="n">
         <v>46</v>
@@ -1083,8 +1125,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
-        <v>3581</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>3581</t>
+        </is>
       </c>
       <c r="B21" t="n">
         <v>40</v>
@@ -1118,8 +1162,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>3582</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>3582</t>
+        </is>
       </c>
       <c r="B22" t="n">
         <v>52</v>
@@ -1153,8 +1199,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>3583</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>3583</t>
+        </is>
       </c>
       <c r="B23" t="n">
         <v>47</v>
@@ -1188,8 +1236,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
-        <v>3584</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>3584</t>
+        </is>
       </c>
       <c r="B24" t="n">
         <v>54</v>
@@ -1223,8 +1273,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>3585</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>3585</t>
+        </is>
       </c>
       <c r="B25" t="n">
         <v>56</v>
@@ -1258,8 +1310,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
-        <v>3586</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3586</t>
+        </is>
       </c>
       <c r="B26" t="n">
         <v>47</v>
@@ -1293,8 +1347,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
-        <v>3587</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>3587</t>
+        </is>
       </c>
       <c r="B27" t="n">
         <v>45</v>
@@ -1326,8 +1382,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>3588</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>3588</t>
+        </is>
       </c>
       <c r="B28" t="n">
         <v>61</v>
@@ -1361,8 +1419,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
-        <v>3589</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>3589</t>
+        </is>
       </c>
       <c r="B29" t="n">
         <v>35</v>
@@ -1396,8 +1456,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
-        <v>3590</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>3590</t>
+        </is>
       </c>
       <c r="B30" t="n">
         <v>44</v>
@@ -1431,8 +1493,10 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
-        <v>3591</v>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>3591</t>
+        </is>
       </c>
       <c r="B31" t="n">
         <v>45</v>
@@ -1466,8 +1530,10 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
-        <v>3592</v>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>3592</t>
+        </is>
       </c>
       <c r="B32" t="n">
         <v>40</v>
@@ -1499,8 +1565,10 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
-        <v>3593</v>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>3593</t>
+        </is>
       </c>
       <c r="B33" t="n">
         <v>52</v>
@@ -1534,8 +1602,10 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
-        <v>3594</v>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>3594</t>
+        </is>
       </c>
       <c r="B34" t="n">
         <v>47</v>
@@ -1569,8 +1639,10 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
-        <v>3595</v>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>3595</t>
+        </is>
       </c>
       <c r="B35" t="n">
         <v>39</v>
@@ -1602,8 +1674,10 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
-        <v>3596</v>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>3596</t>
+        </is>
       </c>
       <c r="B36" t="n">
         <v>44</v>
@@ -1637,8 +1711,10 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
-        <v>3597</v>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>3597</t>
+        </is>
       </c>
       <c r="B37" t="n">
         <v>45</v>
@@ -1672,8 +1748,10 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
-        <v>3598</v>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>3598</t>
+        </is>
       </c>
       <c r="B38" t="n">
         <v>47</v>

</xml_diff>

<commit_message>
Exclui NF 3565 do relatório e do dashboard
Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Lista_vs_Dashboard_Jul.xlsx
+++ b/Comparacao_Lista_vs_Dashboard_Jul.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,10 +474,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>3561</t>
-        </is>
+      <c r="A2" t="n">
+        <v>3561</v>
       </c>
       <c r="B2" t="n">
         <v>13</v>
@@ -515,10 +513,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>3562</t>
-        </is>
+      <c r="A3" t="n">
+        <v>3562</v>
       </c>
       <c r="B3" t="n">
         <v>45</v>
@@ -552,10 +548,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>3564</t>
-        </is>
+      <c r="A4" t="n">
+        <v>3564</v>
       </c>
       <c r="B4" t="n">
         <v>70.73999999999999</v>
@@ -593,20 +587,18 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>3565</t>
-        </is>
+      <c r="A5" t="n">
+        <v>3566</v>
       </c>
       <c r="B5" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SEM_CUSTO</t>
+          <t>CANCELADA</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -616,119 +608,125 @@
       <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>3566</t>
-        </is>
+      <c r="A6" t="n">
+        <v>3567</v>
       </c>
       <c r="B6" t="n">
-        <v>48</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="C6" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="D6" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="E6" t="n">
+        <v>25.24</v>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CANCELADA</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>1007.76</v>
+      </c>
+      <c r="I6" t="n">
+        <v>603.5999999999999</v>
+      </c>
+      <c r="J6" t="n">
+        <v>101.61</v>
+      </c>
+      <c r="K6" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3567</t>
-        </is>
+      <c r="A7" t="n">
+        <v>3568</v>
       </c>
       <c r="B7" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="C7" t="n">
-        <v>34.76</v>
+        <v>45.85</v>
       </c>
       <c r="D7" t="n">
-        <v>34.76</v>
+        <v>45.85</v>
       </c>
       <c r="E7" t="n">
-        <v>25.24</v>
+        <v>0.15</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>CONFERE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>1007.76</v>
+        <v>560.8</v>
       </c>
       <c r="I7" t="n">
-        <v>603.5999999999999</v>
+        <v>332</v>
       </c>
       <c r="J7" t="n">
-        <v>101.61</v>
+        <v>25</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>3568</t>
-        </is>
+      <c r="A8" t="n">
+        <v>3569</v>
       </c>
       <c r="B8" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="C8" t="n">
-        <v>45.85</v>
+        <v>69</v>
       </c>
       <c r="D8" t="n">
-        <v>45.85</v>
+        <v>69</v>
       </c>
       <c r="E8" t="n">
-        <v>0.15</v>
+        <v>7</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CONFERE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>560.8</v>
+        <v>1188</v>
       </c>
       <c r="I8" t="n">
-        <v>332</v>
+        <v>547.6799999999999</v>
       </c>
       <c r="J8" t="n">
-        <v>25</v>
+        <v>153.14</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>3569</t>
-        </is>
+      <c r="A9" t="n">
+        <v>3570</v>
       </c>
       <c r="B9" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C9" t="n">
-        <v>69</v>
+        <v>130.02</v>
       </c>
       <c r="D9" t="n">
-        <v>69</v>
+        <v>130.02</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>100.02</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -737,93 +735,85 @@
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>1188</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="I9" t="n">
-        <v>547.6799999999999</v>
+        <v>18.58</v>
       </c>
       <c r="J9" t="n">
-        <v>153.14</v>
+        <v>25</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>3570</t>
-        </is>
+      <c r="A10" t="n">
+        <v>3571</v>
       </c>
       <c r="B10" t="n">
-        <v>30</v>
-      </c>
-      <c r="C10" t="n">
-        <v>130.02</v>
-      </c>
-      <c r="D10" t="n">
-        <v>130.02</v>
-      </c>
-      <c r="E10" t="n">
-        <v>100.02</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>AUSENTE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="I10" t="n">
-        <v>18.58</v>
-      </c>
-      <c r="J10" t="n">
-        <v>25</v>
-      </c>
-      <c r="K10" t="n">
-        <v>1</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>3571</t>
-        </is>
+      <c r="A11" t="n">
+        <v>3572</v>
       </c>
       <c r="B11" t="n">
-        <v>31</v>
-      </c>
-      <c r="C11" t="inlineStr"/>
+        <v>41</v>
+      </c>
+      <c r="C11" t="n">
+        <v>13.24</v>
+      </c>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>27.76</v>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AUSENTE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>3486.7</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2795.77</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>3572</t>
-        </is>
+      <c r="A12" t="n">
+        <v>3573</v>
       </c>
       <c r="B12" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C12" t="n">
-        <v>13.24</v>
+        <v>37.3</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>27.76</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -832,10 +822,10 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>3486.7</v>
+        <v>718.5599999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>2795.77</v>
+        <v>475.2</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -845,20 +835,20 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>3573</t>
-        </is>
+      <c r="A13" t="n">
+        <v>3574</v>
       </c>
       <c r="B13" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C13" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
+        <v>24.23</v>
+      </c>
+      <c r="D13" t="n">
+        <v>24.23</v>
+      </c>
       <c r="E13" t="n">
-        <v>9.699999999999999</v>
+        <v>19.77</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -867,35 +857,33 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>718.5599999999999</v>
+        <v>2102.4</v>
       </c>
       <c r="I13" t="n">
-        <v>475.2</v>
+        <v>1440</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="K13" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>3574</t>
-        </is>
+      <c r="A14" t="n">
+        <v>3575</v>
       </c>
       <c r="B14" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C14" t="n">
-        <v>24.23</v>
+        <v>24.67</v>
       </c>
       <c r="D14" t="n">
-        <v>24.23</v>
+        <v>24.67</v>
       </c>
       <c r="E14" t="n">
-        <v>19.77</v>
+        <v>33.33</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -904,95 +892,89 @@
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="n">
-        <v>2102.4</v>
+        <v>718.5599999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>1440</v>
+        <v>475.2</v>
       </c>
       <c r="J14" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="K14" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>3575</t>
-        </is>
+      <c r="A15" t="n">
+        <v>3576</v>
       </c>
       <c r="B15" t="n">
-        <v>58</v>
-      </c>
-      <c r="C15" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="D15" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="E15" t="n">
-        <v>33.33</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>AUSENTE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
-        <v>718.5599999999999</v>
-      </c>
-      <c r="I15" t="n">
-        <v>475.2</v>
-      </c>
-      <c r="J15" t="n">
-        <v>60</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>3576</t>
-        </is>
+      <c r="A16" t="n">
+        <v>3577</v>
       </c>
       <c r="B16" t="n">
-        <v>48</v>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+        <v>46</v>
+      </c>
+      <c r="C16" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="D16" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4.62</v>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>AUSENTE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>19820</v>
+      </c>
+      <c r="I16" t="n">
+        <v>12595</v>
+      </c>
+      <c r="J16" t="n">
+        <v>190</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>3577</t>
-        </is>
+      <c r="A17" t="n">
+        <v>3578</v>
       </c>
       <c r="B17" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C17" t="n">
-        <v>41.38</v>
+        <v>34.14</v>
       </c>
       <c r="D17" t="n">
-        <v>41.38</v>
+        <v>34.14</v>
       </c>
       <c r="E17" t="n">
-        <v>4.62</v>
+        <v>18.86</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1001,35 +983,33 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>19820</v>
+        <v>2874.24</v>
       </c>
       <c r="I17" t="n">
-        <v>12595</v>
+        <v>1900.8</v>
       </c>
       <c r="J17" t="n">
-        <v>190</v>
+        <v>60</v>
       </c>
       <c r="K17" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>3578</t>
-        </is>
+      <c r="A18" t="n">
+        <v>3579</v>
       </c>
       <c r="B18" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C18" t="n">
-        <v>34.14</v>
+        <v>61.72</v>
       </c>
       <c r="D18" t="n">
-        <v>34.14</v>
+        <v>51.75</v>
       </c>
       <c r="E18" t="n">
-        <v>18.86</v>
+        <v>11.72</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1038,35 +1018,33 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>2874.24</v>
+        <v>3374.5</v>
       </c>
       <c r="I18" t="n">
-        <v>1900.8</v>
+        <v>1869.94</v>
       </c>
       <c r="J18" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>3579</t>
-        </is>
+      <c r="A19" t="n">
+        <v>3580</v>
       </c>
       <c r="B19" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C19" t="n">
-        <v>61.72</v>
+        <v>108.23</v>
       </c>
       <c r="D19" t="n">
-        <v>51.75</v>
+        <v>108.23</v>
       </c>
       <c r="E19" t="n">
-        <v>11.72</v>
+        <v>62.23</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1075,35 +1053,33 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>3374.5</v>
+        <v>292.8</v>
       </c>
       <c r="I19" t="n">
-        <v>1869.94</v>
+        <v>127.68</v>
       </c>
       <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3581</v>
+      </c>
+      <c r="B20" t="n">
         <v>40</v>
       </c>
-      <c r="K19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>3580</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>46</v>
-      </c>
       <c r="C20" t="n">
-        <v>108.23</v>
+        <v>112.34</v>
       </c>
       <c r="D20" t="n">
-        <v>108.23</v>
+        <v>112.34</v>
       </c>
       <c r="E20" t="n">
-        <v>62.23</v>
+        <v>72.34</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1112,35 +1088,33 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>292.8</v>
+        <v>376</v>
       </c>
       <c r="I20" t="n">
-        <v>127.68</v>
+        <v>133</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="K20" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>3581</t>
-        </is>
+      <c r="A21" t="n">
+        <v>3582</v>
       </c>
       <c r="B21" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C21" t="n">
-        <v>112.34</v>
+        <v>39.05</v>
       </c>
       <c r="D21" t="n">
-        <v>112.34</v>
+        <v>39.05</v>
       </c>
       <c r="E21" t="n">
-        <v>72.34</v>
+        <v>12.95</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1149,35 +1123,33 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>376</v>
+        <v>460</v>
       </c>
       <c r="I21" t="n">
-        <v>133</v>
+        <v>266</v>
       </c>
       <c r="J21" t="n">
-        <v>59</v>
+        <v>47.81</v>
       </c>
       <c r="K21" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>3582</t>
-        </is>
+      <c r="A22" t="n">
+        <v>3583</v>
       </c>
       <c r="B22" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C22" t="n">
-        <v>39.05</v>
+        <v>33.62</v>
       </c>
       <c r="D22" t="n">
-        <v>39.05</v>
+        <v>18.71</v>
       </c>
       <c r="E22" t="n">
-        <v>12.95</v>
+        <v>13.38</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1186,35 +1158,33 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>460</v>
+        <v>3316</v>
       </c>
       <c r="I22" t="n">
-        <v>266</v>
+        <v>2253.38</v>
       </c>
       <c r="J22" t="n">
-        <v>47.81</v>
+        <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>3583</t>
-        </is>
+      <c r="A23" t="n">
+        <v>3584</v>
       </c>
       <c r="B23" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C23" t="n">
-        <v>33.62</v>
+        <v>103.7</v>
       </c>
       <c r="D23" t="n">
-        <v>18.71</v>
+        <v>103.7</v>
       </c>
       <c r="E23" t="n">
-        <v>13.38</v>
+        <v>49.7</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1223,35 +1193,33 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>3316</v>
+        <v>556</v>
       </c>
       <c r="I23" t="n">
-        <v>2253.38</v>
+        <v>228.2</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="K23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>3584</t>
-        </is>
+      <c r="A24" t="n">
+        <v>3585</v>
       </c>
       <c r="B24" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C24" t="n">
-        <v>103.7</v>
+        <v>39.64</v>
       </c>
       <c r="D24" t="n">
-        <v>103.7</v>
+        <v>39.64</v>
       </c>
       <c r="E24" t="n">
-        <v>49.7</v>
+        <v>16.36</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1260,35 +1228,33 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>556</v>
+        <v>1820</v>
       </c>
       <c r="I24" t="n">
-        <v>228.2</v>
+        <v>1162</v>
       </c>
       <c r="J24" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K24" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>3585</t>
-        </is>
+      <c r="A25" t="n">
+        <v>3586</v>
       </c>
       <c r="B25" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C25" t="n">
-        <v>39.64</v>
+        <v>104.6</v>
       </c>
       <c r="D25" t="n">
-        <v>39.64</v>
+        <v>104.6</v>
       </c>
       <c r="E25" t="n">
-        <v>16.36</v>
+        <v>57.6</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1297,35 +1263,31 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>1820</v>
+        <v>704.7</v>
       </c>
       <c r="I25" t="n">
-        <v>1162</v>
+        <v>288.3</v>
       </c>
       <c r="J25" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>3586</t>
-        </is>
+      <c r="A26" t="n">
+        <v>3587</v>
       </c>
       <c r="B26" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C26" t="n">
-        <v>104.6</v>
-      </c>
-      <c r="D26" t="n">
-        <v>104.6</v>
-      </c>
+        <v>16.15</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>57.6</v>
+        <v>28.85</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1334,33 +1296,33 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>704.7</v>
+        <v>1277</v>
       </c>
       <c r="I26" t="n">
-        <v>288.3</v>
+        <v>998.3200000000001</v>
       </c>
       <c r="J26" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>3587</t>
-        </is>
+      <c r="A27" t="n">
+        <v>3588</v>
       </c>
       <c r="B27" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C27" t="n">
-        <v>16.15</v>
-      </c>
-      <c r="D27" t="inlineStr"/>
+        <v>22.73</v>
+      </c>
+      <c r="D27" t="n">
+        <v>40.38</v>
+      </c>
       <c r="E27" t="n">
-        <v>28.85</v>
+        <v>38.27</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1369,35 +1331,33 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>1277</v>
+        <v>10590</v>
       </c>
       <c r="I27" t="n">
-        <v>998.3200000000001</v>
+        <v>7834.799999999999</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>3588</t>
-        </is>
+      <c r="A28" t="n">
+        <v>3589</v>
       </c>
       <c r="B28" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C28" t="n">
-        <v>22.73</v>
+        <v>46.62</v>
       </c>
       <c r="D28" t="n">
-        <v>40.38</v>
+        <v>46.62</v>
       </c>
       <c r="E28" t="n">
-        <v>38.27</v>
+        <v>11.62</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1406,35 +1366,33 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>10590</v>
+        <v>928.36</v>
       </c>
       <c r="I28" t="n">
-        <v>7834.799999999999</v>
+        <v>534</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>3589</t>
-        </is>
+      <c r="A29" t="n">
+        <v>3590</v>
       </c>
       <c r="B29" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C29" t="n">
-        <v>46.62</v>
+        <v>76.84</v>
       </c>
       <c r="D29" t="n">
-        <v>46.62</v>
+        <v>76.84</v>
       </c>
       <c r="E29" t="n">
-        <v>11.62</v>
+        <v>32.84</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1443,35 +1401,33 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>928.36</v>
+        <v>1485</v>
       </c>
       <c r="I29" t="n">
-        <v>534</v>
+        <v>684.6</v>
       </c>
       <c r="J29" t="n">
-        <v>60</v>
+        <v>137.74</v>
       </c>
       <c r="K29" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>3590</t>
-        </is>
+      <c r="A30" t="n">
+        <v>3591</v>
       </c>
       <c r="B30" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C30" t="n">
-        <v>76.84</v>
+        <v>41.68</v>
       </c>
       <c r="D30" t="n">
-        <v>76.84</v>
+        <v>41.68</v>
       </c>
       <c r="E30" t="n">
-        <v>32.84</v>
+        <v>3.32</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1480,35 +1436,31 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>1485</v>
+        <v>1137.12</v>
       </c>
       <c r="I30" t="n">
-        <v>684.6</v>
+        <v>686.4</v>
       </c>
       <c r="J30" t="n">
-        <v>137.74</v>
+        <v>60</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>3591</t>
-        </is>
+      <c r="A31" t="n">
+        <v>3592</v>
       </c>
       <c r="B31" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C31" t="n">
-        <v>41.68</v>
-      </c>
-      <c r="D31" t="n">
-        <v>41.68</v>
-      </c>
+        <v>49.38</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
-        <v>3.32</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1517,33 +1469,33 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>1137.12</v>
+        <v>1017.2</v>
       </c>
       <c r="I31" t="n">
-        <v>686.4</v>
+        <v>578.59</v>
       </c>
       <c r="J31" t="n">
-        <v>60</v>
+        <v>59.34</v>
       </c>
       <c r="K31" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>3592</t>
-        </is>
+      <c r="A32" t="n">
+        <v>3593</v>
       </c>
       <c r="B32" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C32" t="n">
-        <v>49.38</v>
-      </c>
-      <c r="D32" t="inlineStr"/>
+        <v>60.37</v>
+      </c>
+      <c r="D32" t="n">
+        <v>60.37</v>
+      </c>
       <c r="E32" t="n">
-        <v>9.380000000000001</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1552,35 +1504,33 @@
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="n">
-        <v>1017.2</v>
+        <v>1673.28</v>
       </c>
       <c r="I32" t="n">
-        <v>578.59</v>
+        <v>760.3200000000001</v>
       </c>
       <c r="J32" t="n">
-        <v>59.34</v>
+        <v>300</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>3593</t>
-        </is>
+      <c r="A33" t="n">
+        <v>3594</v>
       </c>
       <c r="B33" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C33" t="n">
-        <v>60.37</v>
+        <v>73.59</v>
       </c>
       <c r="D33" t="n">
-        <v>60.37</v>
+        <v>73.59</v>
       </c>
       <c r="E33" t="n">
-        <v>8.369999999999999</v>
+        <v>26.59</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1595,29 +1545,25 @@
         <v>760.3200000000001</v>
       </c>
       <c r="J33" t="n">
-        <v>300</v>
+        <v>199.5</v>
       </c>
       <c r="K33" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>3594</t>
-        </is>
+      <c r="A34" t="n">
+        <v>3595</v>
       </c>
       <c r="B34" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C34" t="n">
-        <v>73.59</v>
-      </c>
-      <c r="D34" t="n">
-        <v>73.59</v>
-      </c>
+        <v>32.94</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="n">
-        <v>26.59</v>
+        <v>6.06</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1626,33 +1572,33 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>1673.28</v>
+        <v>1044.2</v>
       </c>
       <c r="I34" t="n">
-        <v>760.3200000000001</v>
+        <v>679.3399999999999</v>
       </c>
       <c r="J34" t="n">
-        <v>199.5</v>
+        <v>45</v>
       </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>3595</t>
-        </is>
+      <c r="A35" t="n">
+        <v>3596</v>
       </c>
       <c r="B35" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C35" t="n">
-        <v>32.94</v>
-      </c>
-      <c r="D35" t="inlineStr"/>
+        <v>70.73999999999999</v>
+      </c>
+      <c r="D35" t="n">
+        <v>70.73999999999999</v>
+      </c>
       <c r="E35" t="n">
-        <v>6.06</v>
+        <v>26.74</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1661,35 +1607,33 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>1044.2</v>
+        <v>645.36</v>
       </c>
       <c r="I35" t="n">
-        <v>679.3399999999999</v>
+        <v>343.2</v>
       </c>
       <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>3597</v>
+      </c>
+      <c r="B36" t="n">
         <v>45</v>
       </c>
-      <c r="K35" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>3596</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>44</v>
-      </c>
       <c r="C36" t="n">
-        <v>70.73999999999999</v>
+        <v>52.32</v>
       </c>
       <c r="D36" t="n">
-        <v>70.73999999999999</v>
+        <v>52.32</v>
       </c>
       <c r="E36" t="n">
-        <v>26.74</v>
+        <v>7.32</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1698,89 +1642,50 @@
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>645.36</v>
+        <v>1372.5</v>
       </c>
       <c r="I36" t="n">
-        <v>343.2</v>
+        <v>674.13</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>219.41</v>
       </c>
       <c r="K36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>3597</t>
-        </is>
+      <c r="A37" t="n">
+        <v>3598</v>
       </c>
       <c r="B37" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C37" t="n">
-        <v>52.32</v>
+        <v>46.83</v>
       </c>
       <c r="D37" t="n">
-        <v>52.32</v>
+        <v>46.83</v>
       </c>
       <c r="E37" t="n">
-        <v>7.32</v>
+        <v>0.17</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>CONFERE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
-        <v>1372.5</v>
+        <v>2352</v>
       </c>
       <c r="I37" t="n">
-        <v>674.13</v>
+        <v>1372.8</v>
       </c>
       <c r="J37" t="n">
-        <v>219.41</v>
+        <v>120</v>
       </c>
       <c r="K37" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>3598</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>47</v>
-      </c>
-      <c r="C38" t="n">
-        <v>46.83</v>
-      </c>
-      <c r="D38" t="n">
-        <v>46.83</v>
-      </c>
-      <c r="E38" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>CONFERE</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="n">
-        <v>2352</v>
-      </c>
-      <c r="I38" t="n">
-        <v>1372.8</v>
-      </c>
-      <c r="J38" t="n">
-        <v>120</v>
-      </c>
-      <c r="K38" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Exclui NF 3566 do relatório e do dashboard
Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Comparacao_Lista_vs_Dashboard_Jul.xlsx
+++ b/Comparacao_Lista_vs_Dashboard_Jul.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,90 +588,104 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>3566</v>
+        <v>3567</v>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="C5" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="D5" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="E5" t="n">
+        <v>25.24</v>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CANCELADA</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>1007.76</v>
+      </c>
+      <c r="I5" t="n">
+        <v>603.5999999999999</v>
+      </c>
+      <c r="J5" t="n">
+        <v>101.61</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3567</v>
+        <v>3568</v>
       </c>
       <c r="B6" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="C6" t="n">
-        <v>34.76</v>
+        <v>45.85</v>
       </c>
       <c r="D6" t="n">
-        <v>34.76</v>
+        <v>45.85</v>
       </c>
       <c r="E6" t="n">
-        <v>25.24</v>
+        <v>0.15</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>CONFERE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="n">
-        <v>1007.76</v>
+        <v>560.8</v>
       </c>
       <c r="I6" t="n">
-        <v>603.5999999999999</v>
+        <v>332</v>
       </c>
       <c r="J6" t="n">
-        <v>101.61</v>
+        <v>25</v>
       </c>
       <c r="K6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3568</v>
+        <v>3569</v>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="C7" t="n">
-        <v>45.85</v>
+        <v>69</v>
       </c>
       <c r="D7" t="n">
-        <v>45.85</v>
+        <v>69</v>
       </c>
       <c r="E7" t="n">
-        <v>0.15</v>
+        <v>7</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CONFERE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>560.8</v>
+        <v>1188</v>
       </c>
       <c r="I7" t="n">
-        <v>332</v>
+        <v>547.6799999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>25</v>
+        <v>153.14</v>
       </c>
       <c r="K7" t="n">
         <v>1</v>
@@ -679,19 +693,19 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3569</v>
+        <v>3570</v>
       </c>
       <c r="B8" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
-        <v>69</v>
+        <v>130.02</v>
       </c>
       <c r="D8" t="n">
-        <v>69</v>
+        <v>130.02</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>100.02</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -700,13 +714,13 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>1188</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="I8" t="n">
-        <v>547.6799999999999</v>
+        <v>18.58</v>
       </c>
       <c r="J8" t="n">
-        <v>153.14</v>
+        <v>25</v>
       </c>
       <c r="K8" t="n">
         <v>1</v>
@@ -714,73 +728,71 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3570</v>
+        <v>3571</v>
       </c>
       <c r="B9" t="n">
-        <v>30</v>
-      </c>
-      <c r="C9" t="n">
-        <v>130.02</v>
-      </c>
-      <c r="D9" t="n">
-        <v>130.02</v>
-      </c>
-      <c r="E9" t="n">
-        <v>100.02</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>AUSENTE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
-        <v>74.59999999999999</v>
-      </c>
-      <c r="I9" t="n">
-        <v>18.58</v>
-      </c>
-      <c r="J9" t="n">
-        <v>25</v>
-      </c>
-      <c r="K9" t="n">
-        <v>1</v>
-      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>3571</v>
+        <v>3572</v>
       </c>
       <c r="B10" t="n">
-        <v>31</v>
-      </c>
-      <c r="C10" t="inlineStr"/>
+        <v>41</v>
+      </c>
+      <c r="C10" t="n">
+        <v>13.24</v>
+      </c>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>27.76</v>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AUSENTE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>3486.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2795.77</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3572</v>
+        <v>3573</v>
       </c>
       <c r="B11" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C11" t="n">
-        <v>13.24</v>
+        <v>37.3</v>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>27.76</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -789,10 +801,10 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>3486.7</v>
+        <v>718.5599999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>2795.77</v>
+        <v>475.2</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -803,17 +815,19 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3573</v>
+        <v>3574</v>
       </c>
       <c r="B12" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C12" t="n">
-        <v>37.3</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>24.23</v>
+      </c>
+      <c r="D12" t="n">
+        <v>24.23</v>
+      </c>
       <c r="E12" t="n">
-        <v>9.699999999999999</v>
+        <v>19.77</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -822,13 +836,13 @@
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>718.5599999999999</v>
+        <v>2102.4</v>
       </c>
       <c r="I12" t="n">
-        <v>475.2</v>
+        <v>1440</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="K12" t="n">
         <v>1</v>
@@ -836,19 +850,19 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3574</v>
+        <v>3575</v>
       </c>
       <c r="B13" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="C13" t="n">
-        <v>24.23</v>
+        <v>24.67</v>
       </c>
       <c r="D13" t="n">
-        <v>24.23</v>
+        <v>24.67</v>
       </c>
       <c r="E13" t="n">
-        <v>19.77</v>
+        <v>33.33</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -857,13 +871,13 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>2102.4</v>
+        <v>718.5599999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>1440</v>
+        <v>475.2</v>
       </c>
       <c r="J13" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="K13" t="n">
         <v>1</v>
@@ -871,75 +885,75 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3575</v>
+        <v>3576</v>
       </c>
       <c r="B14" t="n">
-        <v>58</v>
-      </c>
-      <c r="C14" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="D14" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="E14" t="n">
-        <v>33.33</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>AUSENTE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
-        <v>718.5599999999999</v>
-      </c>
-      <c r="I14" t="n">
-        <v>475.2</v>
-      </c>
-      <c r="J14" t="n">
-        <v>60</v>
-      </c>
-      <c r="K14" t="n">
-        <v>1</v>
-      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3576</v>
+        <v>3577</v>
       </c>
       <c r="B15" t="n">
-        <v>48</v>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
+        <v>46</v>
+      </c>
+      <c r="C15" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="D15" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.62</v>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AUSENTE</t>
+          <t>DIVERGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>19820</v>
+      </c>
+      <c r="I15" t="n">
+        <v>12595</v>
+      </c>
+      <c r="J15" t="n">
+        <v>190</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>3577</v>
+        <v>3578</v>
       </c>
       <c r="B16" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C16" t="n">
-        <v>41.38</v>
+        <v>34.14</v>
       </c>
       <c r="D16" t="n">
-        <v>41.38</v>
+        <v>34.14</v>
       </c>
       <c r="E16" t="n">
-        <v>4.62</v>
+        <v>18.86</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -948,13 +962,13 @@
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>19820</v>
+        <v>2874.24</v>
       </c>
       <c r="I16" t="n">
-        <v>12595</v>
+        <v>1900.8</v>
       </c>
       <c r="J16" t="n">
-        <v>190</v>
+        <v>60</v>
       </c>
       <c r="K16" t="n">
         <v>1</v>
@@ -962,19 +976,19 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>3578</v>
+        <v>3579</v>
       </c>
       <c r="B17" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C17" t="n">
-        <v>34.14</v>
+        <v>61.72</v>
       </c>
       <c r="D17" t="n">
-        <v>34.14</v>
+        <v>51.75</v>
       </c>
       <c r="E17" t="n">
-        <v>18.86</v>
+        <v>11.72</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -983,33 +997,33 @@
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
-        <v>2874.24</v>
+        <v>3374.5</v>
       </c>
       <c r="I17" t="n">
-        <v>1900.8</v>
+        <v>1869.94</v>
       </c>
       <c r="J17" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>3579</v>
+        <v>3580</v>
       </c>
       <c r="B18" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C18" t="n">
-        <v>61.72</v>
+        <v>108.23</v>
       </c>
       <c r="D18" t="n">
-        <v>51.75</v>
+        <v>108.23</v>
       </c>
       <c r="E18" t="n">
-        <v>11.72</v>
+        <v>62.23</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1018,33 +1032,33 @@
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
-        <v>3374.5</v>
+        <v>292.8</v>
       </c>
       <c r="I18" t="n">
-        <v>1869.94</v>
+        <v>127.68</v>
       </c>
       <c r="J18" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>3580</v>
+        <v>3581</v>
       </c>
       <c r="B19" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C19" t="n">
-        <v>108.23</v>
+        <v>112.34</v>
       </c>
       <c r="D19" t="n">
-        <v>108.23</v>
+        <v>112.34</v>
       </c>
       <c r="E19" t="n">
-        <v>62.23</v>
+        <v>72.34</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1053,13 +1067,13 @@
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
-        <v>292.8</v>
+        <v>376</v>
       </c>
       <c r="I19" t="n">
-        <v>127.68</v>
+        <v>133</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="K19" t="n">
         <v>1</v>
@@ -1067,19 +1081,19 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>3581</v>
+        <v>3582</v>
       </c>
       <c r="B20" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C20" t="n">
-        <v>112.34</v>
+        <v>39.05</v>
       </c>
       <c r="D20" t="n">
-        <v>112.34</v>
+        <v>39.05</v>
       </c>
       <c r="E20" t="n">
-        <v>72.34</v>
+        <v>12.95</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1088,13 +1102,13 @@
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>376</v>
+        <v>460</v>
       </c>
       <c r="I20" t="n">
-        <v>133</v>
+        <v>266</v>
       </c>
       <c r="J20" t="n">
-        <v>59</v>
+        <v>47.81</v>
       </c>
       <c r="K20" t="n">
         <v>1</v>
@@ -1102,19 +1116,19 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>3582</v>
+        <v>3583</v>
       </c>
       <c r="B21" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C21" t="n">
-        <v>39.05</v>
+        <v>33.62</v>
       </c>
       <c r="D21" t="n">
-        <v>39.05</v>
+        <v>18.71</v>
       </c>
       <c r="E21" t="n">
-        <v>12.95</v>
+        <v>13.38</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1123,33 +1137,33 @@
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>460</v>
+        <v>3316</v>
       </c>
       <c r="I21" t="n">
-        <v>266</v>
+        <v>2253.38</v>
       </c>
       <c r="J21" t="n">
-        <v>47.81</v>
+        <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="B22" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C22" t="n">
-        <v>33.62</v>
+        <v>103.7</v>
       </c>
       <c r="D22" t="n">
-        <v>18.71</v>
+        <v>103.7</v>
       </c>
       <c r="E22" t="n">
-        <v>13.38</v>
+        <v>49.7</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1158,33 +1172,33 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>3316</v>
+        <v>556</v>
       </c>
       <c r="I22" t="n">
-        <v>2253.38</v>
+        <v>228.2</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="K22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>3584</v>
+        <v>3585</v>
       </c>
       <c r="B23" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C23" t="n">
-        <v>103.7</v>
+        <v>39.64</v>
       </c>
       <c r="D23" t="n">
-        <v>103.7</v>
+        <v>39.64</v>
       </c>
       <c r="E23" t="n">
-        <v>49.7</v>
+        <v>16.36</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1193,13 +1207,13 @@
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
-        <v>556</v>
+        <v>1820</v>
       </c>
       <c r="I23" t="n">
-        <v>228.2</v>
+        <v>1162</v>
       </c>
       <c r="J23" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K23" t="n">
         <v>1</v>
@@ -1207,19 +1221,19 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>3585</v>
+        <v>3586</v>
       </c>
       <c r="B24" t="n">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C24" t="n">
-        <v>39.64</v>
+        <v>104.6</v>
       </c>
       <c r="D24" t="n">
-        <v>39.64</v>
+        <v>104.6</v>
       </c>
       <c r="E24" t="n">
-        <v>16.36</v>
+        <v>57.6</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1228,13 +1242,13 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="n">
-        <v>1820</v>
+        <v>704.7</v>
       </c>
       <c r="I24" t="n">
-        <v>1162</v>
+        <v>288.3</v>
       </c>
       <c r="J24" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K24" t="n">
         <v>1</v>
@@ -1242,19 +1256,17 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>3586</v>
+        <v>3587</v>
       </c>
       <c r="B25" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C25" t="n">
-        <v>104.6</v>
-      </c>
-      <c r="D25" t="n">
-        <v>104.6</v>
-      </c>
+        <v>16.15</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>57.6</v>
+        <v>28.85</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1263,13 +1275,13 @@
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="n">
-        <v>704.7</v>
+        <v>1277</v>
       </c>
       <c r="I25" t="n">
-        <v>288.3</v>
+        <v>998.3200000000001</v>
       </c>
       <c r="J25" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -1277,17 +1289,19 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3587</v>
+        <v>3588</v>
       </c>
       <c r="B26" t="n">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C26" t="n">
-        <v>16.15</v>
-      </c>
-      <c r="D26" t="inlineStr"/>
+        <v>22.73</v>
+      </c>
+      <c r="D26" t="n">
+        <v>40.38</v>
+      </c>
       <c r="E26" t="n">
-        <v>28.85</v>
+        <v>38.27</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1296,33 +1310,33 @@
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="n">
-        <v>1277</v>
+        <v>10590</v>
       </c>
       <c r="I26" t="n">
-        <v>998.3200000000001</v>
+        <v>7834.799999999999</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3588</v>
+        <v>3589</v>
       </c>
       <c r="B27" t="n">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C27" t="n">
-        <v>22.73</v>
+        <v>46.62</v>
       </c>
       <c r="D27" t="n">
-        <v>40.38</v>
+        <v>46.62</v>
       </c>
       <c r="E27" t="n">
-        <v>38.27</v>
+        <v>11.62</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1331,33 +1345,33 @@
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>10590</v>
+        <v>928.36</v>
       </c>
       <c r="I27" t="n">
-        <v>7834.799999999999</v>
+        <v>534</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3589</v>
+        <v>3590</v>
       </c>
       <c r="B28" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C28" t="n">
-        <v>46.62</v>
+        <v>76.84</v>
       </c>
       <c r="D28" t="n">
-        <v>46.62</v>
+        <v>76.84</v>
       </c>
       <c r="E28" t="n">
-        <v>11.62</v>
+        <v>32.84</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1366,13 +1380,13 @@
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
-        <v>928.36</v>
+        <v>1485</v>
       </c>
       <c r="I28" t="n">
-        <v>534</v>
+        <v>684.6</v>
       </c>
       <c r="J28" t="n">
-        <v>60</v>
+        <v>137.74</v>
       </c>
       <c r="K28" t="n">
         <v>1</v>
@@ -1380,19 +1394,19 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>3590</v>
+        <v>3591</v>
       </c>
       <c r="B29" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C29" t="n">
-        <v>76.84</v>
+        <v>41.68</v>
       </c>
       <c r="D29" t="n">
-        <v>76.84</v>
+        <v>41.68</v>
       </c>
       <c r="E29" t="n">
-        <v>32.84</v>
+        <v>3.32</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1401,13 +1415,13 @@
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="n">
-        <v>1485</v>
+        <v>1137.12</v>
       </c>
       <c r="I29" t="n">
-        <v>684.6</v>
+        <v>686.4</v>
       </c>
       <c r="J29" t="n">
-        <v>137.74</v>
+        <v>60</v>
       </c>
       <c r="K29" t="n">
         <v>1</v>
@@ -1415,19 +1429,17 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>3591</v>
+        <v>3592</v>
       </c>
       <c r="B30" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C30" t="n">
-        <v>41.68</v>
-      </c>
-      <c r="D30" t="n">
-        <v>41.68</v>
-      </c>
+        <v>49.38</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="n">
-        <v>3.32</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1436,13 +1448,13 @@
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="n">
-        <v>1137.12</v>
+        <v>1017.2</v>
       </c>
       <c r="I30" t="n">
-        <v>686.4</v>
+        <v>578.59</v>
       </c>
       <c r="J30" t="n">
-        <v>60</v>
+        <v>59.34</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
@@ -1450,17 +1462,19 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3592</v>
+        <v>3593</v>
       </c>
       <c r="B31" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C31" t="n">
-        <v>49.38</v>
-      </c>
-      <c r="D31" t="inlineStr"/>
+        <v>60.37</v>
+      </c>
+      <c r="D31" t="n">
+        <v>60.37</v>
+      </c>
       <c r="E31" t="n">
-        <v>9.380000000000001</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1469,13 +1483,13 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="n">
-        <v>1017.2</v>
+        <v>1673.28</v>
       </c>
       <c r="I31" t="n">
-        <v>578.59</v>
+        <v>760.3200000000001</v>
       </c>
       <c r="J31" t="n">
-        <v>59.34</v>
+        <v>300</v>
       </c>
       <c r="K31" t="n">
         <v>1</v>
@@ -1483,19 +1497,19 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>3593</v>
+        <v>3594</v>
       </c>
       <c r="B32" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C32" t="n">
-        <v>60.37</v>
+        <v>73.59</v>
       </c>
       <c r="D32" t="n">
-        <v>60.37</v>
+        <v>73.59</v>
       </c>
       <c r="E32" t="n">
-        <v>8.369999999999999</v>
+        <v>26.59</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1510,7 +1524,7 @@
         <v>760.3200000000001</v>
       </c>
       <c r="J32" t="n">
-        <v>300</v>
+        <v>199.5</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
@@ -1518,19 +1532,17 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3594</v>
+        <v>3595</v>
       </c>
       <c r="B33" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C33" t="n">
-        <v>73.59</v>
-      </c>
-      <c r="D33" t="n">
-        <v>73.59</v>
-      </c>
+        <v>32.94</v>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>26.59</v>
+        <v>6.06</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1539,31 +1551,33 @@
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
-        <v>1673.28</v>
+        <v>1044.2</v>
       </c>
       <c r="I33" t="n">
-        <v>760.3200000000001</v>
+        <v>679.3399999999999</v>
       </c>
       <c r="J33" t="n">
-        <v>199.5</v>
+        <v>45</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3595</v>
+        <v>3596</v>
       </c>
       <c r="B34" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C34" t="n">
-        <v>32.94</v>
-      </c>
-      <c r="D34" t="inlineStr"/>
+        <v>70.73999999999999</v>
+      </c>
+      <c r="D34" t="n">
+        <v>70.73999999999999</v>
+      </c>
       <c r="E34" t="n">
-        <v>6.06</v>
+        <v>26.74</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1572,33 +1586,33 @@
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
-        <v>1044.2</v>
+        <v>645.36</v>
       </c>
       <c r="I34" t="n">
-        <v>679.3399999999999</v>
+        <v>343.2</v>
       </c>
       <c r="J34" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3596</v>
+        <v>3597</v>
       </c>
       <c r="B35" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C35" t="n">
-        <v>70.73999999999999</v>
+        <v>52.32</v>
       </c>
       <c r="D35" t="n">
-        <v>70.73999999999999</v>
+        <v>52.32</v>
       </c>
       <c r="E35" t="n">
-        <v>26.74</v>
+        <v>7.32</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1607,85 +1621,50 @@
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
-        <v>645.36</v>
+        <v>1372.5</v>
       </c>
       <c r="I35" t="n">
-        <v>343.2</v>
+        <v>674.13</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>219.41</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3597</v>
+        <v>3598</v>
       </c>
       <c r="B36" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C36" t="n">
-        <v>52.32</v>
+        <v>46.83</v>
       </c>
       <c r="D36" t="n">
-        <v>52.32</v>
+        <v>46.83</v>
       </c>
       <c r="E36" t="n">
-        <v>7.32</v>
+        <v>0.17</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>DIVERGE</t>
+          <t>CONFERE</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>1372.5</v>
+        <v>2352</v>
       </c>
       <c r="I36" t="n">
-        <v>674.13</v>
+        <v>1372.8</v>
       </c>
       <c r="J36" t="n">
-        <v>219.41</v>
+        <v>120</v>
       </c>
       <c r="K36" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>3598</v>
-      </c>
-      <c r="B37" t="n">
-        <v>47</v>
-      </c>
-      <c r="C37" t="n">
-        <v>46.83</v>
-      </c>
-      <c r="D37" t="n">
-        <v>46.83</v>
-      </c>
-      <c r="E37" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>CONFERE</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="n">
-        <v>2352</v>
-      </c>
-      <c r="I37" t="n">
-        <v>1372.8</v>
-      </c>
-      <c r="J37" t="n">
-        <v>120</v>
-      </c>
-      <c r="K37" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>